<commit_message>
Add cross-report consistency check, browser discovery for all 15 reports, and dedupe Unilever cash-flow line
</commit_message>
<xml_diff>
--- a/outputs/019f8d79-c13d-7a22-850f-fed24fc926c0/FiscalAI_Financial_Statements.xlsx
+++ b/outputs/019f8d79-c13d-7a22-850f-fed24fc926c0/FiscalAI_Financial_Statements.xlsx
@@ -11758,7 +11758,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K62"/>
+  <dimension ref="A1:K61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="85" customWidth="1" min="1" max="1"/>
@@ -11911,7 +11911,9 @@
           <t>Share of net profit of joint ventures/associates and other (income)/loss from non- current investments</t>
         </is>
       </c>
-      <c r="B6" s="29" t="n"/>
+      <c r="B6" s="29" t="n">
+        <v>-231</v>
+      </c>
       <c r="C6" s="29" t="n">
         <v>-173</v>
       </c>
@@ -12645,470 +12647,472 @@
       <c r="K28" s="29" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="28" t="inlineStr">
-        <is>
-          <t>Share of net profit of joint ventures/associates and other income/(loss) from non-current investments and associates</t>
-        </is>
-      </c>
-      <c r="B29" s="29" t="n">
-        <v>-231</v>
-      </c>
-      <c r="C29" s="29" t="n">
-        <v>-173</v>
-      </c>
-      <c r="D29" s="29" t="n"/>
-      <c r="E29" s="29" t="n"/>
-      <c r="F29" s="29" t="n"/>
-      <c r="G29" s="29" t="n"/>
-      <c r="H29" s="29" t="n"/>
-      <c r="I29" s="29" t="n"/>
-      <c r="J29" s="29" t="n"/>
-      <c r="K29" s="29" t="n"/>
+      <c r="A29" s="30" t="inlineStr">
+        <is>
+          <t>Total cash flows from operating activities</t>
+        </is>
+      </c>
+      <c r="B29" s="31" t="n">
+        <v>7047</v>
+      </c>
+      <c r="C29" s="31" t="n">
+        <v>7879</v>
+      </c>
+      <c r="D29" s="31" t="n">
+        <v>7318</v>
+      </c>
+      <c r="E29" s="31" t="n">
+        <v>8109</v>
+      </c>
+      <c r="F29" s="31" t="n">
+        <v>9058</v>
+      </c>
+      <c r="G29" s="31" t="n">
+        <v>7972</v>
+      </c>
+      <c r="H29" s="31" t="n">
+        <v>7282</v>
+      </c>
+      <c r="I29" s="31" t="n">
+        <v>9426</v>
+      </c>
+      <c r="J29" s="31" t="n">
+        <v>9519</v>
+      </c>
+      <c r="K29" s="31" t="n">
+        <v>8350</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="30" t="inlineStr">
         <is>
-          <t>Total cash flows from operating activities</t>
+          <t>Cash flow from operating activities</t>
         </is>
       </c>
       <c r="B30" s="31" t="n">
-        <v>7047</v>
+        <v>9298</v>
       </c>
       <c r="C30" s="31" t="n">
-        <v>7879</v>
+        <v>10043</v>
       </c>
       <c r="D30" s="31" t="n">
-        <v>7318</v>
+        <v>9612</v>
       </c>
       <c r="E30" s="31" t="n">
-        <v>8109</v>
+        <v>10641</v>
       </c>
       <c r="F30" s="31" t="n">
-        <v>9058</v>
+        <v>10933</v>
       </c>
       <c r="G30" s="31" t="n">
-        <v>7972</v>
+        <v>10305</v>
       </c>
       <c r="H30" s="31" t="n">
-        <v>7282</v>
+        <v>10089</v>
       </c>
       <c r="I30" s="31" t="n">
-        <v>9426</v>
-      </c>
-      <c r="J30" s="31" t="n">
-        <v>9519</v>
-      </c>
-      <c r="K30" s="31" t="n">
-        <v>8350</v>
-      </c>
+        <v>11561</v>
+      </c>
+      <c r="J30" s="31" t="n"/>
+      <c r="K30" s="31" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="30" t="inlineStr">
-        <is>
-          <t>Cash flow from operating activities</t>
-        </is>
-      </c>
-      <c r="B31" s="31" t="n">
-        <v>9298</v>
-      </c>
-      <c r="C31" s="31" t="n">
-        <v>10043</v>
-      </c>
-      <c r="D31" s="31" t="n">
-        <v>9612</v>
-      </c>
-      <c r="E31" s="31" t="n">
-        <v>10641</v>
-      </c>
-      <c r="F31" s="31" t="n">
-        <v>10933</v>
-      </c>
-      <c r="G31" s="31" t="n">
-        <v>10305</v>
-      </c>
-      <c r="H31" s="31" t="n">
-        <v>10089</v>
-      </c>
-      <c r="I31" s="31" t="n">
-        <v>11561</v>
-      </c>
-      <c r="J31" s="31" t="n"/>
-      <c r="K31" s="31" t="n"/>
+      <c r="A31" s="28" t="inlineStr">
+        <is>
+          <t>Elimination of losses/(profits) on disposals</t>
+        </is>
+      </c>
+      <c r="B31" s="29" t="n">
+        <v>127</v>
+      </c>
+      <c r="C31" s="29" t="n">
+        <v>-298</v>
+      </c>
+      <c r="D31" s="29" t="n">
+        <v>-4313</v>
+      </c>
+      <c r="E31" s="29" t="n">
+        <v>60</v>
+      </c>
+      <c r="F31" s="29" t="n">
+        <v>60</v>
+      </c>
+      <c r="G31" s="29" t="n">
+        <v>23</v>
+      </c>
+      <c r="H31" s="29" t="n">
+        <v>-2335</v>
+      </c>
+      <c r="I31" s="29" t="n">
+        <v>-440</v>
+      </c>
+      <c r="J31" s="29" t="n">
+        <v>259</v>
+      </c>
+      <c r="K31" s="29" t="n">
+        <v>58</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="28" t="inlineStr">
         <is>
-          <t>Elimination of losses/(profits) on disposals</t>
+          <t>Purchase of intangible assets</t>
         </is>
       </c>
       <c r="B32" s="29" t="n">
-        <v>127</v>
+        <v>-232</v>
       </c>
       <c r="C32" s="29" t="n">
-        <v>-298</v>
+        <v>-158</v>
       </c>
       <c r="D32" s="29" t="n">
-        <v>-4313</v>
+        <v>-203</v>
       </c>
       <c r="E32" s="29" t="n">
-        <v>60</v>
+        <v>-210</v>
       </c>
       <c r="F32" s="29" t="n">
-        <v>60</v>
+        <v>-158</v>
       </c>
       <c r="G32" s="29" t="n">
-        <v>23</v>
+        <v>-232</v>
       </c>
       <c r="H32" s="29" t="n">
-        <v>-2335</v>
+        <v>-253</v>
       </c>
       <c r="I32" s="29" t="n">
-        <v>-440</v>
+        <v>-241</v>
       </c>
       <c r="J32" s="29" t="n">
-        <v>259</v>
+        <v>-233</v>
       </c>
       <c r="K32" s="29" t="n">
-        <v>58</v>
+        <v>-174</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="28" t="inlineStr">
         <is>
-          <t>Purchase of intangible assets</t>
+          <t>Purchase of property, plant and equipment</t>
         </is>
       </c>
       <c r="B33" s="29" t="n">
-        <v>-232</v>
+        <v>-1804</v>
       </c>
       <c r="C33" s="29" t="n">
-        <v>-158</v>
+        <v>-1509</v>
       </c>
       <c r="D33" s="29" t="n">
-        <v>-203</v>
+        <v>-1329</v>
       </c>
       <c r="E33" s="29" t="n">
-        <v>-210</v>
+        <v>-1316</v>
       </c>
       <c r="F33" s="29" t="n">
-        <v>-158</v>
+        <v>-863</v>
       </c>
       <c r="G33" s="29" t="n">
-        <v>-232</v>
+        <v>-1108</v>
       </c>
       <c r="H33" s="29" t="n">
-        <v>-253</v>
+        <v>-1456</v>
       </c>
       <c r="I33" s="29" t="n">
-        <v>-241</v>
+        <v>-1194</v>
       </c>
       <c r="J33" s="29" t="n">
-        <v>-233</v>
+        <v>-1381</v>
       </c>
       <c r="K33" s="29" t="n">
-        <v>-174</v>
+        <v>-1417</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="28" t="inlineStr">
         <is>
-          <t>Purchase of property, plant and equipment</t>
+          <t>Disposal of property, plant and equipment</t>
         </is>
       </c>
       <c r="B34" s="29" t="n">
-        <v>-1804</v>
+        <v>158</v>
       </c>
       <c r="C34" s="29" t="n">
-        <v>-1509</v>
+        <v>46</v>
       </c>
       <c r="D34" s="29" t="n">
-        <v>-1329</v>
+        <v>108</v>
       </c>
       <c r="E34" s="29" t="n">
-        <v>-1316</v>
+        <v>97</v>
       </c>
       <c r="F34" s="29" t="n">
-        <v>-863</v>
+        <v>89</v>
       </c>
       <c r="G34" s="29" t="n">
-        <v>-1108</v>
+        <v>101</v>
       </c>
       <c r="H34" s="29" t="n">
-        <v>-1456</v>
+        <v>82</v>
       </c>
       <c r="I34" s="29" t="n">
-        <v>-1194</v>
+        <v>15</v>
       </c>
       <c r="J34" s="29" t="n">
-        <v>-1381</v>
+        <v>15</v>
       </c>
       <c r="K34" s="29" t="n">
-        <v>-1417</v>
+        <v>126</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="28" t="inlineStr">
         <is>
-          <t>Disposal of property, plant and equipment</t>
+          <t>Acquisition of businesses and investments in joint ventures and associates</t>
         </is>
       </c>
       <c r="B35" s="29" t="n">
-        <v>158</v>
+        <v>-1731</v>
       </c>
       <c r="C35" s="29" t="n">
-        <v>46</v>
+        <v>-4896</v>
       </c>
       <c r="D35" s="29" t="n">
-        <v>108</v>
+        <v>-1336</v>
       </c>
       <c r="E35" s="29" t="n">
-        <v>97</v>
+        <v>-1122</v>
       </c>
       <c r="F35" s="29" t="n">
-        <v>89</v>
+        <v>-1426</v>
       </c>
       <c r="G35" s="29" t="n">
-        <v>101</v>
+        <v>-2131</v>
       </c>
       <c r="H35" s="29" t="n">
-        <v>82</v>
+        <v>-979</v>
       </c>
       <c r="I35" s="29" t="n">
-        <v>15</v>
+        <v>-100</v>
       </c>
       <c r="J35" s="29" t="n">
-        <v>15</v>
+        <v>-734</v>
       </c>
       <c r="K35" s="29" t="n">
-        <v>126</v>
+        <v>-1674</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="28" t="inlineStr">
         <is>
-          <t>Acquisition of businesses and investments in joint ventures and associates</t>
+          <t>Disposal of businesses, joint ventures and associates</t>
         </is>
       </c>
       <c r="B36" s="29" t="n">
-        <v>-1731</v>
+        <v>30</v>
       </c>
       <c r="C36" s="29" t="n">
-        <v>-4896</v>
+        <v>561</v>
       </c>
       <c r="D36" s="29" t="n">
-        <v>-1336</v>
+        <v>7093</v>
       </c>
       <c r="E36" s="29" t="n">
-        <v>-1122</v>
+        <v>177</v>
       </c>
       <c r="F36" s="29" t="n">
-        <v>-1426</v>
+        <v>39</v>
       </c>
       <c r="G36" s="29" t="n">
-        <v>-2131</v>
+        <v>43</v>
       </c>
       <c r="H36" s="29" t="n">
-        <v>-979</v>
+        <v>4622</v>
       </c>
       <c r="I36" s="29" t="n">
-        <v>-100</v>
+        <v>436</v>
       </c>
       <c r="J36" s="29" t="n">
-        <v>-734</v>
+        <v>910</v>
       </c>
       <c r="K36" s="29" t="n">
-        <v>-1674</v>
+        <v>107</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="28" t="inlineStr">
         <is>
-          <t>Disposal of businesses, joint ventures and associates</t>
+          <t>Acquisition of other non-current investments</t>
         </is>
       </c>
       <c r="B37" s="29" t="n">
-        <v>30</v>
+        <v>-208</v>
       </c>
       <c r="C37" s="29" t="n">
-        <v>561</v>
+        <v>-317</v>
       </c>
       <c r="D37" s="29" t="n">
-        <v>7093</v>
+        <v>-94</v>
       </c>
       <c r="E37" s="29" t="n">
-        <v>177</v>
+        <v>-160</v>
       </c>
       <c r="F37" s="29" t="n">
-        <v>39</v>
+        <v>-128</v>
       </c>
       <c r="G37" s="29" t="n">
-        <v>43</v>
+        <v>-142</v>
       </c>
       <c r="H37" s="29" t="n">
-        <v>4622</v>
+        <v>-170</v>
       </c>
       <c r="I37" s="29" t="n">
-        <v>436</v>
+        <v>-533</v>
       </c>
       <c r="J37" s="29" t="n">
-        <v>910</v>
+        <v>-166</v>
       </c>
       <c r="K37" s="29" t="n">
-        <v>107</v>
+        <v>-111</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="28" t="inlineStr">
         <is>
-          <t>Acquisition of other non-current investments</t>
+          <t>Disposal of other non-current investments</t>
         </is>
       </c>
       <c r="B38" s="29" t="n">
-        <v>-208</v>
+        <v>173</v>
       </c>
       <c r="C38" s="29" t="n">
-        <v>-317</v>
+        <v>251</v>
       </c>
       <c r="D38" s="29" t="n">
-        <v>-94</v>
+        <v>151</v>
       </c>
       <c r="E38" s="29" t="n">
-        <v>-160</v>
+        <v>55</v>
       </c>
       <c r="F38" s="29" t="n">
-        <v>-128</v>
+        <v>51</v>
       </c>
       <c r="G38" s="29" t="n">
-        <v>-142</v>
+        <v>137</v>
       </c>
       <c r="H38" s="29" t="n">
-        <v>-170</v>
+        <v>266</v>
       </c>
       <c r="I38" s="29" t="n">
-        <v>-533</v>
+        <v>62</v>
       </c>
       <c r="J38" s="29" t="n">
-        <v>-166</v>
+        <v>59</v>
       </c>
       <c r="K38" s="29" t="n">
-        <v>-111</v>
+        <v>239</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="28" t="inlineStr">
         <is>
-          <t>Disposal of other non-current investments</t>
+          <t>Dividends from joint ventures, associates and other non-current investments</t>
         </is>
       </c>
       <c r="B39" s="29" t="n">
-        <v>173</v>
+        <v>186</v>
       </c>
       <c r="C39" s="29" t="n">
-        <v>251</v>
+        <v>138</v>
       </c>
       <c r="D39" s="29" t="n">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="E39" s="29" t="n">
-        <v>55</v>
+        <v>164</v>
       </c>
       <c r="F39" s="29" t="n">
-        <v>51</v>
+        <v>188</v>
       </c>
       <c r="G39" s="29" t="n">
-        <v>137</v>
+        <v>185</v>
       </c>
       <c r="H39" s="29" t="n">
-        <v>266</v>
+        <v>185</v>
       </c>
       <c r="I39" s="29" t="n">
-        <v>62</v>
+        <v>239</v>
       </c>
       <c r="J39" s="29" t="n">
-        <v>59</v>
+        <v>261</v>
       </c>
       <c r="K39" s="29" t="n">
-        <v>239</v>
+        <v>243</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="28" t="inlineStr">
         <is>
-          <t>Dividends from joint ventures, associates and other non-current investments</t>
+          <t>Sale/(purchase) of financial assets</t>
         </is>
       </c>
       <c r="B40" s="29" t="n">
-        <v>186</v>
+        <v>135</v>
       </c>
       <c r="C40" s="29" t="n">
-        <v>138</v>
+        <v>-149</v>
       </c>
       <c r="D40" s="29" t="n">
-        <v>154</v>
+        <v>-10</v>
       </c>
       <c r="E40" s="29" t="n">
-        <v>164</v>
+        <v>-68</v>
       </c>
       <c r="F40" s="29" t="n">
-        <v>188</v>
+        <v>558</v>
       </c>
       <c r="G40" s="29" t="n">
-        <v>185</v>
+        <v>-247</v>
       </c>
       <c r="H40" s="29" t="n">
-        <v>185</v>
+        <v>-131</v>
       </c>
       <c r="I40" s="29" t="n">
-        <v>239</v>
+        <v>-318</v>
       </c>
       <c r="J40" s="29" t="n">
-        <v>261</v>
+        <v>476</v>
       </c>
       <c r="K40" s="29" t="n">
-        <v>243</v>
+        <v>-85</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="28" t="inlineStr">
         <is>
-          <t>Sale/(purchase) of financial assets</t>
-        </is>
-      </c>
-      <c r="B41" s="29" t="n">
-        <v>135</v>
-      </c>
-      <c r="C41" s="29" t="n">
-        <v>-149</v>
-      </c>
-      <c r="D41" s="29" t="n">
-        <v>-10</v>
-      </c>
-      <c r="E41" s="29" t="n">
-        <v>-68</v>
-      </c>
-      <c r="F41" s="29" t="n">
-        <v>558</v>
-      </c>
-      <c r="G41" s="29" t="n">
-        <v>-247</v>
-      </c>
-      <c r="H41" s="29" t="n">
-        <v>-131</v>
-      </c>
+          <t>Net cash flow used in continuing investing activities</t>
+        </is>
+      </c>
+      <c r="B41" s="29" t="n"/>
+      <c r="C41" s="29" t="n"/>
+      <c r="D41" s="29" t="n"/>
+      <c r="E41" s="29" t="n"/>
+      <c r="F41" s="29" t="n"/>
+      <c r="G41" s="29" t="n"/>
+      <c r="H41" s="29" t="n"/>
       <c r="I41" s="29" t="n">
-        <v>-318</v>
+        <v>-1411</v>
       </c>
       <c r="J41" s="29" t="n">
-        <v>476</v>
+        <v>-423</v>
       </c>
       <c r="K41" s="29" t="n">
-        <v>-85</v>
+        <v>-2394</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="28" t="inlineStr">
         <is>
-          <t>Net cash flow used in continuing investing activities</t>
+          <t>Net investing cash flows attributable to discontinued operations</t>
         </is>
       </c>
       <c r="B42" s="29" t="n"/>
@@ -13119,379 +13123,379 @@
       <c r="G42" s="29" t="n"/>
       <c r="H42" s="29" t="n"/>
       <c r="I42" s="29" t="n">
-        <v>-1411</v>
+        <v>-883</v>
       </c>
       <c r="J42" s="29" t="n">
-        <v>-423</v>
+        <v>-202</v>
       </c>
       <c r="K42" s="29" t="n">
-        <v>-2394</v>
+        <v>-724</v>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="28" t="inlineStr">
-        <is>
-          <t>Net investing cash flows attributable to discontinued operations</t>
-        </is>
-      </c>
-      <c r="B43" s="29" t="n"/>
-      <c r="C43" s="29" t="n"/>
-      <c r="D43" s="29" t="n"/>
-      <c r="E43" s="29" t="n"/>
-      <c r="F43" s="29" t="n"/>
-      <c r="G43" s="29" t="n"/>
-      <c r="H43" s="29" t="n"/>
-      <c r="I43" s="29" t="n">
-        <v>-883</v>
-      </c>
-      <c r="J43" s="29" t="n">
-        <v>-202</v>
-      </c>
-      <c r="K43" s="29" t="n">
-        <v>-724</v>
+      <c r="A43" s="30" t="inlineStr">
+        <is>
+          <t>Total cash outflow used in investing activities</t>
+        </is>
+      </c>
+      <c r="B43" s="31" t="n">
+        <v>-3188</v>
+      </c>
+      <c r="C43" s="31" t="n">
+        <v>-5879</v>
+      </c>
+      <c r="D43" s="31" t="n">
+        <v>4644</v>
+      </c>
+      <c r="E43" s="31" t="n">
+        <v>-2237</v>
+      </c>
+      <c r="F43" s="31" t="n">
+        <v>-1481</v>
+      </c>
+      <c r="G43" s="31" t="n">
+        <v>-3246</v>
+      </c>
+      <c r="H43" s="31" t="n">
+        <v>2453</v>
+      </c>
+      <c r="I43" s="31" t="n">
+        <v>-2294</v>
+      </c>
+      <c r="J43" s="31" t="n">
+        <v>-625</v>
+      </c>
+      <c r="K43" s="31" t="n">
+        <v>-3118</v>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="30" t="inlineStr">
-        <is>
-          <t>Total cash outflow used in investing activities</t>
-        </is>
-      </c>
-      <c r="B44" s="31" t="n">
-        <v>-3188</v>
-      </c>
-      <c r="C44" s="31" t="n">
-        <v>-5879</v>
-      </c>
-      <c r="D44" s="31" t="n">
-        <v>4644</v>
-      </c>
-      <c r="E44" s="31" t="n">
-        <v>-2237</v>
-      </c>
-      <c r="F44" s="31" t="n">
-        <v>-1481</v>
-      </c>
-      <c r="G44" s="31" t="n">
-        <v>-3246</v>
-      </c>
-      <c r="H44" s="31" t="n">
-        <v>2453</v>
-      </c>
-      <c r="I44" s="31" t="n">
-        <v>-2294</v>
-      </c>
-      <c r="J44" s="31" t="n">
-        <v>-625</v>
-      </c>
-      <c r="K44" s="31" t="n">
-        <v>-3118</v>
+      <c r="A44" s="28" t="inlineStr">
+        <is>
+          <t>Dividends paid on ordinary share capital</t>
+        </is>
+      </c>
+      <c r="B44" s="29" t="n">
+        <v>-3609</v>
+      </c>
+      <c r="C44" s="29" t="n">
+        <v>-3916</v>
+      </c>
+      <c r="D44" s="29" t="n">
+        <v>-4066</v>
+      </c>
+      <c r="E44" s="29" t="n">
+        <v>-4209</v>
+      </c>
+      <c r="F44" s="29" t="n">
+        <v>-4279</v>
+      </c>
+      <c r="G44" s="29" t="n">
+        <v>-4483</v>
+      </c>
+      <c r="H44" s="29" t="n">
+        <v>-4329</v>
+      </c>
+      <c r="I44" s="29" t="n">
+        <v>-4363</v>
+      </c>
+      <c r="J44" s="29" t="n">
+        <v>-4319</v>
+      </c>
+      <c r="K44" s="29" t="n">
+        <v>-4453</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="28" t="inlineStr">
         <is>
-          <t>Dividends paid on ordinary share capital</t>
-        </is>
-      </c>
-      <c r="B45" s="29" t="n">
-        <v>-3609</v>
-      </c>
+          <t>Interest paid</t>
+        </is>
+      </c>
+      <c r="B45" s="29" t="n"/>
       <c r="C45" s="29" t="n">
-        <v>-3916</v>
+        <v>-574</v>
       </c>
       <c r="D45" s="29" t="n">
-        <v>-4066</v>
+        <v>-571</v>
       </c>
       <c r="E45" s="29" t="n">
-        <v>-4209</v>
+        <v>-694</v>
       </c>
       <c r="F45" s="29" t="n">
-        <v>-4279</v>
+        <v>-624</v>
       </c>
       <c r="G45" s="29" t="n">
-        <v>-4483</v>
+        <v>-488</v>
       </c>
       <c r="H45" s="29" t="n">
-        <v>-4329</v>
+        <v>-744</v>
       </c>
       <c r="I45" s="29" t="n">
-        <v>-4363</v>
+        <v>-751</v>
       </c>
       <c r="J45" s="29" t="n">
-        <v>-4319</v>
+        <v>-929</v>
       </c>
       <c r="K45" s="29" t="n">
-        <v>-4453</v>
+        <v>-1018</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="28" t="inlineStr">
         <is>
-          <t>Interest paid</t>
-        </is>
-      </c>
-      <c r="B46" s="29" t="n"/>
+          <t>Net change in short-term borrowings</t>
+        </is>
+      </c>
+      <c r="B46" s="29" t="n">
+        <v>258</v>
+      </c>
       <c r="C46" s="29" t="n">
-        <v>-574</v>
+        <v>2695</v>
       </c>
       <c r="D46" s="29" t="n">
-        <v>-571</v>
+        <v>-4026</v>
       </c>
       <c r="E46" s="29" t="n">
-        <v>-694</v>
+        <v>337</v>
       </c>
       <c r="F46" s="29" t="n">
-        <v>-624</v>
+        <v>722</v>
       </c>
       <c r="G46" s="29" t="n">
-        <v>-488</v>
+        <v>656</v>
       </c>
       <c r="H46" s="29" t="n">
-        <v>-744</v>
+        <v>-545</v>
       </c>
       <c r="I46" s="29" t="n">
-        <v>-751</v>
+        <v>-506</v>
       </c>
       <c r="J46" s="29" t="n">
-        <v>-929</v>
+        <v>575</v>
       </c>
       <c r="K46" s="29" t="n">
-        <v>-1018</v>
+        <v>-2228</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="28" t="inlineStr">
         <is>
-          <t>Net change in short-term borrowings</t>
+          <t>Additional financial liabilities</t>
         </is>
       </c>
       <c r="B47" s="29" t="n">
-        <v>258</v>
+        <v>6761</v>
       </c>
       <c r="C47" s="29" t="n">
-        <v>2695</v>
+        <v>8851</v>
       </c>
       <c r="D47" s="29" t="n">
-        <v>-4026</v>
+        <v>10595</v>
       </c>
       <c r="E47" s="29" t="n">
-        <v>337</v>
+        <v>5911</v>
       </c>
       <c r="F47" s="29" t="n">
-        <v>722</v>
+        <v>3117</v>
       </c>
       <c r="G47" s="29" t="n">
-        <v>656</v>
+        <v>4748</v>
       </c>
       <c r="H47" s="29" t="n">
-        <v>-545</v>
+        <v>7776</v>
       </c>
       <c r="I47" s="29" t="n">
-        <v>-506</v>
+        <v>4418</v>
       </c>
       <c r="J47" s="29" t="n">
-        <v>575</v>
+        <v>4234</v>
       </c>
       <c r="K47" s="29" t="n">
-        <v>-2228</v>
+        <v>4278</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="28" t="inlineStr">
         <is>
-          <t>Additional financial liabilities</t>
+          <t>Repayment of financial liabilities</t>
         </is>
       </c>
       <c r="B48" s="29" t="n">
-        <v>6761</v>
+        <v>-5213</v>
       </c>
       <c r="C48" s="29" t="n">
-        <v>8851</v>
+        <v>-2604</v>
       </c>
       <c r="D48" s="29" t="n">
-        <v>10595</v>
+        <v>-6594</v>
       </c>
       <c r="E48" s="29" t="n">
-        <v>5911</v>
+        <v>-4912</v>
       </c>
       <c r="F48" s="29" t="n">
-        <v>3117</v>
+        <v>-3577</v>
       </c>
       <c r="G48" s="29" t="n">
-        <v>4748</v>
+        <v>-3550</v>
       </c>
       <c r="H48" s="29" t="n">
-        <v>7776</v>
+        <v>-8440</v>
       </c>
       <c r="I48" s="29" t="n">
-        <v>4418</v>
+        <v>-3470</v>
       </c>
       <c r="J48" s="29" t="n">
-        <v>4234</v>
+        <v>-3846</v>
       </c>
       <c r="K48" s="29" t="n">
-        <v>4278</v>
+        <v>-3547</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="28" t="inlineStr">
         <is>
-          <t>Repayment of financial liabilities</t>
+          <t>Capital element of lease rental payments</t>
         </is>
       </c>
       <c r="B49" s="29" t="n">
-        <v>-5213</v>
+        <v>-35</v>
       </c>
       <c r="C49" s="29" t="n">
-        <v>-2604</v>
+        <v>-497</v>
       </c>
       <c r="D49" s="29" t="n">
-        <v>-6594</v>
+        <v>-481</v>
       </c>
       <c r="E49" s="29" t="n">
-        <v>-4912</v>
+        <v>-435</v>
       </c>
       <c r="F49" s="29" t="n">
-        <v>-3577</v>
+        <v>-443</v>
       </c>
       <c r="G49" s="29" t="n">
-        <v>-3550</v>
+        <v>-464</v>
       </c>
       <c r="H49" s="29" t="n">
-        <v>-8440</v>
+        <v>-518</v>
       </c>
       <c r="I49" s="29" t="n">
-        <v>-3470</v>
+        <v>-349</v>
       </c>
       <c r="J49" s="29" t="n">
-        <v>-3846</v>
+        <v>-342</v>
       </c>
       <c r="K49" s="29" t="n">
-        <v>-3547</v>
+        <v>-301</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="28" t="inlineStr">
         <is>
-          <t>Capital element of lease rental payments</t>
-        </is>
-      </c>
-      <c r="B50" s="29" t="n">
-        <v>-35</v>
+          <t>Repurchase of shares</t>
+        </is>
+      </c>
+      <c r="B50" s="29" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="C50" s="29" t="n">
-        <v>-497</v>
+        <v>-5014</v>
       </c>
       <c r="D50" s="29" t="n">
-        <v>-481</v>
-      </c>
-      <c r="E50" s="29" t="n">
-        <v>-435</v>
-      </c>
-      <c r="F50" s="29" t="n">
-        <v>-443</v>
+        <v>-6020</v>
+      </c>
+      <c r="E50" s="29" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F50" s="29" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="G50" s="29" t="n">
-        <v>-464</v>
+        <v>-3018</v>
       </c>
       <c r="H50" s="29" t="n">
-        <v>-518</v>
+        <v>-1509</v>
       </c>
       <c r="I50" s="29" t="n">
-        <v>-349</v>
+        <v>-1507</v>
       </c>
       <c r="J50" s="29" t="n">
-        <v>-342</v>
+        <v>-1508</v>
       </c>
       <c r="K50" s="29" t="n">
-        <v>-301</v>
+        <v>-1510</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="28" t="inlineStr">
         <is>
-          <t>Repurchase of shares</t>
-        </is>
-      </c>
-      <c r="B51" s="29" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>Other financing activities(c)</t>
+        </is>
+      </c>
+      <c r="B51" s="29" t="n">
+        <v>-506</v>
       </c>
       <c r="C51" s="29" t="n">
-        <v>-5014</v>
+        <v>-309</v>
       </c>
       <c r="D51" s="29" t="n">
-        <v>-6020</v>
-      </c>
-      <c r="E51" s="29" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F51" s="29" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>-693</v>
+      </c>
+      <c r="E51" s="29" t="n">
+        <v>-464</v>
+      </c>
+      <c r="F51" s="29" t="n">
+        <v>-720</v>
       </c>
       <c r="G51" s="29" t="n">
-        <v>-3018</v>
+        <v>-500</v>
       </c>
       <c r="H51" s="29" t="n">
-        <v>-1509</v>
+        <v>-581</v>
       </c>
       <c r="I51" s="29" t="n">
-        <v>-1507</v>
+        <v>-556</v>
       </c>
       <c r="J51" s="29" t="n">
-        <v>-1508</v>
+        <v>-694</v>
       </c>
       <c r="K51" s="29" t="n">
-        <v>-1510</v>
+        <v>-1105</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="28" t="inlineStr">
         <is>
-          <t>Other financing activities(c)</t>
-        </is>
-      </c>
-      <c r="B52" s="29" t="n">
-        <v>-506</v>
-      </c>
-      <c r="C52" s="29" t="n">
-        <v>-309</v>
-      </c>
-      <c r="D52" s="29" t="n">
-        <v>-693</v>
-      </c>
-      <c r="E52" s="29" t="n">
-        <v>-464</v>
-      </c>
-      <c r="F52" s="29" t="n">
-        <v>-720</v>
-      </c>
-      <c r="G52" s="29" t="n">
-        <v>-500</v>
-      </c>
-      <c r="H52" s="29" t="n">
-        <v>-581</v>
-      </c>
+          <t>Net cash flow used in continuing financing activities</t>
+        </is>
+      </c>
+      <c r="B52" s="29" t="n"/>
+      <c r="C52" s="29" t="n"/>
+      <c r="D52" s="29" t="n"/>
+      <c r="E52" s="29" t="n"/>
+      <c r="F52" s="29" t="n"/>
+      <c r="G52" s="29" t="n"/>
+      <c r="H52" s="29" t="n"/>
       <c r="I52" s="29" t="n">
-        <v>-556</v>
+        <v>-7084</v>
       </c>
       <c r="J52" s="29" t="n">
-        <v>-694</v>
+        <v>-6829</v>
       </c>
       <c r="K52" s="29" t="n">
-        <v>-1105</v>
+        <v>-9884</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="28" t="inlineStr">
         <is>
-          <t>Net cash flow used in continuing financing activities</t>
+          <t>Net financing cash flows attributable to discontinued operations</t>
         </is>
       </c>
       <c r="B53" s="29" t="n"/>
@@ -13502,66 +13506,74 @@
       <c r="G53" s="29" t="n"/>
       <c r="H53" s="29" t="n"/>
       <c r="I53" s="29" t="n">
-        <v>-7084</v>
+        <v>-109</v>
       </c>
       <c r="J53" s="29" t="n">
-        <v>-6829</v>
+        <v>-112</v>
       </c>
       <c r="K53" s="29" t="n">
-        <v>-9884</v>
+        <v>3070</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="28" t="inlineStr">
         <is>
-          <t>Net financing cash flows attributable to discontinued operations</t>
-        </is>
-      </c>
-      <c r="B54" s="29" t="n"/>
-      <c r="C54" s="29" t="n"/>
-      <c r="D54" s="29" t="n"/>
-      <c r="E54" s="29" t="n"/>
-      <c r="F54" s="29" t="n"/>
-      <c r="G54" s="29" t="n"/>
+          <t>Other movements on treasury shares</t>
+        </is>
+      </c>
+      <c r="B54" s="29" t="n">
+        <v>-257</v>
+      </c>
+      <c r="C54" s="29" t="n">
+        <v>-204</v>
+      </c>
+      <c r="D54" s="29" t="n">
+        <v>-257</v>
+      </c>
+      <c r="E54" s="29" t="n">
+        <v>-201</v>
+      </c>
+      <c r="F54" s="29" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G54" s="29" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="H54" s="29" t="n"/>
-      <c r="I54" s="29" t="n">
-        <v>-109</v>
-      </c>
-      <c r="J54" s="29" t="n">
-        <v>-112</v>
-      </c>
-      <c r="K54" s="29" t="n">
-        <v>3070</v>
-      </c>
+      <c r="I54" s="29" t="n"/>
+      <c r="J54" s="29" t="n"/>
+      <c r="K54" s="29" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="28" t="inlineStr">
         <is>
-          <t>Other movements on treasury shares</t>
-        </is>
-      </c>
-      <c r="B55" s="29" t="n">
-        <v>-257</v>
+          <t>Buyback of preference shares</t>
+        </is>
+      </c>
+      <c r="B55" s="29" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="C55" s="29" t="n">
-        <v>-204</v>
-      </c>
-      <c r="D55" s="29" t="n">
-        <v>-257</v>
-      </c>
-      <c r="E55" s="29" t="n">
-        <v>-201</v>
-      </c>
-      <c r="F55" s="29" t="inlineStr">
+        <v>-448</v>
+      </c>
+      <c r="D55" s="29" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G55" s="29" t="inlineStr">
+      <c r="E55" s="29" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
+      <c r="F55" s="29" t="n"/>
+      <c r="G55" s="29" t="n"/>
       <c r="H55" s="29" t="n"/>
       <c r="I55" s="29" t="n"/>
       <c r="J55" s="29" t="n"/>
@@ -13570,27 +13582,17 @@
     <row r="56">
       <c r="A56" s="28" t="inlineStr">
         <is>
-          <t>Buyback of preference shares</t>
-        </is>
-      </c>
-      <c r="B56" s="29" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>Interest and preference dividends paid</t>
+        </is>
+      </c>
+      <c r="B56" s="29" t="n">
+        <v>-472</v>
       </c>
       <c r="C56" s="29" t="n">
-        <v>-448</v>
-      </c>
-      <c r="D56" s="29" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E56" s="29" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+        <v>-470</v>
+      </c>
+      <c r="D56" s="29" t="n"/>
+      <c r="E56" s="29" t="n"/>
       <c r="F56" s="29" t="n"/>
       <c r="G56" s="29" t="n"/>
       <c r="H56" s="29" t="n"/>
@@ -13599,208 +13601,187 @@
       <c r="K56" s="29" t="n"/>
     </row>
     <row r="57">
-      <c r="A57" s="28" t="inlineStr">
-        <is>
-          <t>Interest and preference dividends paid</t>
-        </is>
-      </c>
-      <c r="B57" s="29" t="n">
-        <v>-472</v>
-      </c>
-      <c r="C57" s="29" t="n">
-        <v>-470</v>
-      </c>
-      <c r="D57" s="29" t="n"/>
-      <c r="E57" s="29" t="n"/>
-      <c r="F57" s="29" t="n"/>
-      <c r="G57" s="29" t="n"/>
-      <c r="H57" s="29" t="n"/>
-      <c r="I57" s="29" t="n"/>
-      <c r="J57" s="29" t="n"/>
-      <c r="K57" s="29" t="n"/>
+      <c r="A57" s="30" t="inlineStr">
+        <is>
+          <t>Total cash flow used in financing activities</t>
+        </is>
+      </c>
+      <c r="B57" s="31" t="n">
+        <v>-3073</v>
+      </c>
+      <c r="C57" s="31" t="n">
+        <v>-2020</v>
+      </c>
+      <c r="D57" s="31" t="n">
+        <v>-12113</v>
+      </c>
+      <c r="E57" s="31" t="n">
+        <v>-4667</v>
+      </c>
+      <c r="F57" s="31" t="n">
+        <v>-5804</v>
+      </c>
+      <c r="G57" s="31" t="n">
+        <v>-7099</v>
+      </c>
+      <c r="H57" s="31" t="n">
+        <v>-8890</v>
+      </c>
+      <c r="I57" s="31" t="n">
+        <v>-7193</v>
+      </c>
+      <c r="J57" s="31" t="n">
+        <v>-6941</v>
+      </c>
+      <c r="K57" s="31" t="n">
+        <v>-6814</v>
+      </c>
     </row>
     <row r="58">
-      <c r="A58" s="30" t="inlineStr">
-        <is>
-          <t>Total cash flow used in financing activities</t>
-        </is>
-      </c>
-      <c r="B58" s="31" t="n">
-        <v>-3073</v>
-      </c>
-      <c r="C58" s="31" t="n">
-        <v>-2020</v>
-      </c>
-      <c r="D58" s="31" t="n">
-        <v>-12113</v>
-      </c>
-      <c r="E58" s="31" t="n">
-        <v>-4667</v>
-      </c>
-      <c r="F58" s="31" t="n">
-        <v>-5804</v>
-      </c>
-      <c r="G58" s="31" t="n">
-        <v>-7099</v>
-      </c>
-      <c r="H58" s="31" t="n">
-        <v>-8890</v>
-      </c>
-      <c r="I58" s="31" t="n">
-        <v>-7193</v>
-      </c>
-      <c r="J58" s="31" t="n">
-        <v>-6941</v>
-      </c>
-      <c r="K58" s="31" t="n">
-        <v>-6814</v>
+      <c r="A58" s="28" t="inlineStr">
+        <is>
+          <t>Cash and cash equivalents at the beginning of the year</t>
+        </is>
+      </c>
+      <c r="B58" s="29" t="n">
+        <v>2128</v>
+      </c>
+      <c r="C58" s="29" t="n">
+        <v>3198</v>
+      </c>
+      <c r="D58" s="29" t="n">
+        <v>3169</v>
+      </c>
+      <c r="E58" s="29" t="n">
+        <v>3090</v>
+      </c>
+      <c r="F58" s="29" t="n">
+        <v>4116</v>
+      </c>
+      <c r="G58" s="29" t="n">
+        <v>5475</v>
+      </c>
+      <c r="H58" s="29" t="n">
+        <v>3387</v>
+      </c>
+      <c r="I58" s="29" t="n">
+        <v>4225</v>
+      </c>
+      <c r="J58" s="29" t="n">
+        <v>4045</v>
+      </c>
+      <c r="K58" s="29" t="n">
+        <v>5950</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="28" t="inlineStr">
         <is>
-          <t>Cash and cash equivalents at the beginning of the year</t>
+          <t>Net increase/(decrease) in cash and cash equivalents</t>
         </is>
       </c>
       <c r="B59" s="29" t="n">
-        <v>2128</v>
+        <v>786</v>
       </c>
       <c r="C59" s="29" t="n">
-        <v>3198</v>
+        <v>-20</v>
       </c>
       <c r="D59" s="29" t="n">
-        <v>3169</v>
+        <v>-151</v>
       </c>
       <c r="E59" s="29" t="n">
-        <v>3090</v>
+        <v>1205</v>
       </c>
       <c r="F59" s="29" t="n">
-        <v>4116</v>
+        <v>1773</v>
       </c>
       <c r="G59" s="29" t="n">
-        <v>5475</v>
+        <v>-2373</v>
       </c>
       <c r="H59" s="29" t="n">
-        <v>3387</v>
+        <v>845</v>
       </c>
       <c r="I59" s="29" t="n">
-        <v>4225</v>
+        <v>-61</v>
       </c>
       <c r="J59" s="29" t="n">
-        <v>4045</v>
+        <v>1953</v>
       </c>
       <c r="K59" s="29" t="n">
-        <v>5950</v>
+        <v>-1582</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="28" t="inlineStr">
         <is>
-          <t>Net increase/(decrease) in cash and cash equivalents</t>
+          <t>Effect of foreign exchange rate changes</t>
         </is>
       </c>
       <c r="B60" s="29" t="n">
-        <v>786</v>
+        <v>284</v>
       </c>
       <c r="C60" s="29" t="n">
-        <v>-20</v>
+        <v>-9</v>
       </c>
       <c r="D60" s="29" t="n">
-        <v>-151</v>
+        <v>72</v>
       </c>
       <c r="E60" s="29" t="n">
-        <v>1205</v>
+        <v>-179</v>
       </c>
       <c r="F60" s="29" t="n">
-        <v>1773</v>
+        <v>-414</v>
       </c>
       <c r="G60" s="29" t="n">
-        <v>-2373</v>
+        <v>285</v>
       </c>
       <c r="H60" s="29" t="n">
-        <v>845</v>
+        <v>-7</v>
       </c>
       <c r="I60" s="29" t="n">
-        <v>-61</v>
+        <v>-119</v>
       </c>
       <c r="J60" s="29" t="n">
-        <v>1953</v>
+        <v>-48</v>
       </c>
       <c r="K60" s="29" t="n">
-        <v>-1582</v>
+        <v>-498</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="28" t="inlineStr">
         <is>
-          <t>Effect of foreign exchange rate changes</t>
+          <t>Cash and cash equivalents at the end of the year</t>
         </is>
       </c>
       <c r="B61" s="29" t="n">
-        <v>284</v>
+        <v>3198</v>
       </c>
       <c r="C61" s="29" t="n">
-        <v>-9</v>
+        <v>3169</v>
       </c>
       <c r="D61" s="29" t="n">
-        <v>72</v>
+        <v>3090</v>
       </c>
       <c r="E61" s="29" t="n">
-        <v>-179</v>
+        <v>4116</v>
       </c>
       <c r="F61" s="29" t="n">
-        <v>-414</v>
+        <v>5475</v>
       </c>
       <c r="G61" s="29" t="n">
-        <v>285</v>
+        <v>3387</v>
       </c>
       <c r="H61" s="29" t="n">
-        <v>-7</v>
+        <v>4225</v>
       </c>
       <c r="I61" s="29" t="n">
-        <v>-119</v>
+        <v>4045</v>
       </c>
       <c r="J61" s="29" t="n">
-        <v>-48</v>
+        <v>5950</v>
       </c>
       <c r="K61" s="29" t="n">
-        <v>-498</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="28" t="inlineStr">
-        <is>
-          <t>Cash and cash equivalents at the end of the year</t>
-        </is>
-      </c>
-      <c r="B62" s="29" t="n">
-        <v>3198</v>
-      </c>
-      <c r="C62" s="29" t="n">
-        <v>3169</v>
-      </c>
-      <c r="D62" s="29" t="n">
-        <v>3090</v>
-      </c>
-      <c r="E62" s="29" t="n">
-        <v>4116</v>
-      </c>
-      <c r="F62" s="29" t="n">
-        <v>5475</v>
-      </c>
-      <c r="G62" s="29" t="n">
-        <v>3387</v>
-      </c>
-      <c r="H62" s="29" t="n">
-        <v>4225</v>
-      </c>
-      <c r="I62" s="29" t="n">
-        <v>4045</v>
-      </c>
-      <c r="J62" s="29" t="n">
-        <v>5950</v>
-      </c>
-      <c r="K62" s="29" t="n">
         <v>3870</v>
       </c>
     </row>

</xml_diff>